<commit_message>
Deployed ebea0b16 with MkDocs version: 1.6.0
</commit_message>
<xml_diff>
--- a/Manual/source/tab/connectors.xlsx
+++ b/Manual/source/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="48"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
@@ -1238,6 +1238,15 @@
     <t xml:space="preserve">Analogová zem</t>
   </si>
   <si>
+    <t xml:space="preserve">PT1000_2+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vstup pro 2. PT1000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT1000_2-</t>
+  </si>
+  <si>
     <t xml:space="preserve">PT1000_1+</t>
   </si>
   <si>
@@ -1245,15 +1254,6 @@
   </si>
   <si>
     <t xml:space="preserve">PT1000_1-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PT1000_2+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vstup pro 2. PT1000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PT1000_2-</t>
   </si>
   <si>
     <t xml:space="preserve">DITTL1</t>

</xml_diff>

<commit_message>
Deployed 11510b44 with MkDocs version: 1.6.0
</commit_message>
<xml_diff>
--- a/Manual/source/tab/connectors.xlsx
+++ b/Manual/source/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="48"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="19"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1756" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="445">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller B2CF se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_B2CF“</t>
   </si>
@@ -819,6 +819,9 @@
   </si>
   <si>
     <t xml:space="preserve">0,13 ~ 2,5 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+B2</t>
   </si>
   <si>
     <t xml:space="preserve">+ Brzda motor 2</t>
@@ -7909,12 +7912,11 @@
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="str">
-        <f aca="false">+B2</f>
-        <v>-B2</v>
+      <c r="B3" s="1" t="s">
+        <v>237</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>236</v>
@@ -7928,7 +7930,7 @@
         <v>225</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>236</v>
@@ -7942,7 +7944,7 @@
         <v>226</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>236</v>
@@ -7953,10 +7955,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>236</v>
@@ -7967,10 +7969,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>236</v>
@@ -8026,10 +8028,10 @@
         <v>115</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8037,13 +8039,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8057,7 +8059,7 @@
         <v>120</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8071,7 +8073,7 @@
         <v>111</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8085,7 +8087,7 @@
         <v>114</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -8135,10 +8137,10 @@
         <v>115</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8146,13 +8148,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8163,10 +8165,10 @@
         <v>226</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8177,10 +8179,10 @@
         <v>225</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -8230,10 +8232,10 @@
         <v>173</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8244,10 +8246,10 @@
         <v>173</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8258,10 +8260,10 @@
         <v>173</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8272,10 +8274,10 @@
         <v>119</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -8322,13 +8324,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8336,13 +8338,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -8394,7 +8396,7 @@
         <v>205</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8408,7 +8410,7 @@
         <v>208</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8422,7 +8424,7 @@
         <v>210</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8436,7 +8438,7 @@
         <v>212</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8450,7 +8452,7 @@
         <v>214</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8464,7 +8466,7 @@
         <v>216</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8527,10 +8529,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>206</v>
@@ -8541,10 +8543,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>206</v>
@@ -8555,10 +8557,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>206</v>
@@ -8569,10 +8571,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>206</v>
@@ -8583,10 +8585,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>206</v>
@@ -8597,10 +8599,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>206</v>
@@ -8611,7 +8613,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>210</v>
@@ -8625,10 +8627,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>206</v>
@@ -8639,10 +8641,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>206</v>
@@ -8695,10 +8697,10 @@
         <v>121</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8712,7 +8714,7 @@
         <v>125</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8726,7 +8728,7 @@
         <v>210</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -8778,7 +8780,7 @@
         <v>205</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8792,7 +8794,7 @@
         <v>208</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8806,7 +8808,7 @@
         <v>210</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8820,7 +8822,7 @@
         <v>212</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8834,7 +8836,7 @@
         <v>214</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8848,7 +8850,7 @@
         <v>216</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8911,10 +8913,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>206</v>
@@ -8925,10 +8927,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>206</v>
@@ -8939,10 +8941,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>206</v>
@@ -8953,10 +8955,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>206</v>
@@ -8967,10 +8969,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>206</v>
@@ -8981,10 +8983,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>206</v>
@@ -8995,10 +8997,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>206</v>
@@ -9009,10 +9011,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>206</v>
@@ -9023,7 +9025,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>210</v>
@@ -9037,10 +9039,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>206</v>
@@ -9051,10 +9053,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>206</v>
@@ -9211,13 +9213,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9225,13 +9227,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9504,10 +9506,10 @@
         <v>204</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9518,10 +9520,10 @@
         <v>207</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9529,13 +9531,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9543,13 +9545,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9601,10 +9603,10 @@
         <v>204</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9615,10 +9617,10 @@
         <v>207</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9626,13 +9628,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9640,13 +9642,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9707,10 +9709,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>123</v>
@@ -9721,10 +9723,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>123</v>
@@ -9773,13 +9775,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9787,13 +9789,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9801,13 +9803,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9815,13 +9817,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9829,13 +9831,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9843,13 +9845,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9857,13 +9859,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9871,13 +9873,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9936,10 +9938,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>112</v>
@@ -9950,10 +9952,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>112</v>
@@ -9964,10 +9966,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>112</v>
@@ -9978,10 +9980,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>112</v>
@@ -10031,13 +10033,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10045,13 +10047,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10059,13 +10061,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10073,13 +10075,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -10122,7 +10124,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>166</v>
@@ -10133,7 +10135,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>164</v>
@@ -10144,7 +10146,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>162</v>
@@ -10155,7 +10157,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>160</v>
@@ -10166,7 +10168,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>158</v>
@@ -10177,7 +10179,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>156</v>
@@ -10188,7 +10190,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>154</v>
@@ -10199,7 +10201,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>152</v>
@@ -10210,10 +10212,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10221,10 +10223,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10337,7 +10339,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>166</v>
@@ -10348,7 +10350,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>164</v>
@@ -10359,7 +10361,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>162</v>
@@ -10370,7 +10372,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>160</v>
@@ -10381,7 +10383,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>158</v>
@@ -10392,7 +10394,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>156</v>
@@ -10403,7 +10405,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>154</v>
@@ -10414,7 +10416,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>152</v>
@@ -10425,10 +10427,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10436,10 +10438,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10477,10 +10479,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>108</v>
@@ -10488,24 +10490,24 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10584,10 +10586,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>112</v>
@@ -10598,10 +10600,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>112</v>
@@ -10615,7 +10617,7 @@
         <v>115</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>112</v>
@@ -10934,7 +10936,7 @@
         <v>182</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11067,7 +11069,7 @@
         <v>183</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11109,7 +11111,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>59</v>
@@ -11118,7 +11120,7 @@
         <v>200</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11126,7 +11128,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>59</v>
@@ -11135,7 +11137,7 @@
         <v>198</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11143,7 +11145,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>192</v>
@@ -11152,7 +11154,7 @@
         <v>196</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11160,7 +11162,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>191</v>
@@ -11169,7 +11171,7 @@
         <v>194</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11220,7 +11222,7 @@
         <v>190</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11237,7 +11239,7 @@
         <v>188</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11316,7 +11318,7 @@
         <v>183</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11358,7 +11360,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>59</v>
@@ -11367,7 +11369,7 @@
         <v>200</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11375,7 +11377,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>59</v>
@@ -11384,7 +11386,7 @@
         <v>198</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11392,7 +11394,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>192</v>
@@ -11401,7 +11403,7 @@
         <v>196</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11409,7 +11411,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>191</v>
@@ -11418,7 +11420,7 @@
         <v>194</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11531,7 +11533,7 @@
         <v>183</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11573,7 +11575,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>59</v>
@@ -11582,7 +11584,7 @@
         <v>200</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11590,7 +11592,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>59</v>
@@ -11599,7 +11601,7 @@
         <v>198</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11607,7 +11609,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>192</v>
@@ -11616,7 +11618,7 @@
         <v>196</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11624,7 +11626,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>191</v>
@@ -11633,7 +11635,7 @@
         <v>194</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11747,10 +11749,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11761,7 +11763,7 @@
         <v>126</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11769,10 +11771,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11780,10 +11782,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>378</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11791,10 +11793,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11802,10 +11804,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>381</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11813,10 +11815,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11827,7 +11829,7 @@
         <v>149</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11835,10 +11837,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11849,7 +11851,7 @@
         <v>149</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11857,10 +11859,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11871,7 +11873,7 @@
         <v>149</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12265,7 +12267,7 @@
         <v>165</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12276,7 +12278,7 @@
         <v>163</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12287,7 +12289,7 @@
         <v>161</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12298,7 +12300,7 @@
         <v>159</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12309,7 +12311,7 @@
         <v>157</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12320,7 +12322,7 @@
         <v>155</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12331,7 +12333,7 @@
         <v>153</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12342,7 +12344,7 @@
         <v>151</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12350,10 +12352,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12361,10 +12363,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12372,10 +12374,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12383,10 +12385,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12397,7 +12399,7 @@
         <v>143</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12408,7 +12410,7 @@
         <v>141</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12419,7 +12421,7 @@
         <v>139</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12430,7 +12432,7 @@
         <v>137</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12441,7 +12443,7 @@
         <v>135</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12452,7 +12454,7 @@
         <v>133</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -12495,10 +12497,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12506,10 +12508,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12517,10 +12519,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12528,10 +12530,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12539,10 +12541,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12550,10 +12552,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12561,10 +12563,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12572,10 +12574,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -12618,10 +12620,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12629,10 +12631,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12640,10 +12642,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12651,10 +12653,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12662,10 +12664,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12676,7 +12678,7 @@
         <v>119</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12684,10 +12686,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12695,10 +12697,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12706,10 +12708,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12717,10 +12719,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12772,10 +12774,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12783,10 +12785,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12794,10 +12796,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12805,10 +12807,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12816,10 +12818,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12827,10 +12829,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12838,10 +12840,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12849,10 +12851,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Deployed 9b83985a with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Manual/source/tab/connectors.xlsx
+++ b/Manual/source/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="59"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="60"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
@@ -68,6 +68,10 @@
     <sheet name="X6_TGS560_50_DCbus" sheetId="58" state="visible" r:id="rId60"/>
     <sheet name="X4_TGS560_24V_5pin_BCZ" sheetId="59" state="visible" r:id="rId61"/>
     <sheet name="S1_TGS560_DIP" sheetId="60" state="visible" r:id="rId62"/>
+    <sheet name="LED_TGS560" sheetId="61" state="visible" r:id="rId63"/>
+    <sheet name="X4_ACIN_4pin_TGS560_25" sheetId="62" state="visible" r:id="rId64"/>
+    <sheet name="X1_DC_6pin_TGS560_25" sheetId="63" state="visible" r:id="rId65"/>
+    <sheet name="X5_RBR_3pin_TGS560_25" sheetId="64" state="visible" r:id="rId66"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -79,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2037" uniqueCount="492">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller B2CF se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_B2CF“</t>
   </si>
@@ -1533,19 +1537,64 @@
     <t xml:space="preserve">0001</t>
   </si>
   <si>
+    <t xml:space="preserve">Zvolený 4 bit. kód</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Význam – volba funkce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">výchozí nastavení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rezervováno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Červená LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Počet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Význam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">krátké bliknutí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">podpětí Dcbus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">přepětí Dcbus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chyba fázového napětí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vysoká interní teplota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vysoká teplota softstart modulu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vysoká teplota brzdného rezistoru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelená LED</t>
+  </si>
+  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">Zvolený 4 bit. kód</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Význam – volba funkce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brzdný odpor interní</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brzdný odpor 1 kW</t>
+    <t xml:space="preserve">trvalý svit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zařízení připraveno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trvale vypnuto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zařízení nepřipraveno</t>
   </si>
 </sst>
 </file>
@@ -1705,11 +1754,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -14613,7 +14662,7 @@
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
@@ -14674,23 +14723,12 @@
         <v>471</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>472</v>
-      </c>
-    </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>473</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14698,7 +14736,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="H8" s="14"/>
       <c r="I8" s="13"/>
@@ -14708,7 +14746,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H9" s="14"/>
       <c r="I9" s="13"/>
@@ -14718,7 +14756,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="13"/>
@@ -14728,7 +14766,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="13"/>
@@ -14738,7 +14776,7 @@
         <v>100</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H12" s="14"/>
       <c r="I12" s="13"/>
@@ -14748,7 +14786,7 @@
         <v>101</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="13"/>
@@ -14758,7 +14796,7 @@
         <v>110</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H14" s="14"/>
       <c r="I14" s="13"/>
@@ -14768,7 +14806,7 @@
         <v>111</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H15" s="14"/>
       <c r="I15" s="13"/>
@@ -14778,7 +14816,7 @@
         <v>1000</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H16" s="14"/>
       <c r="I16" s="13"/>
@@ -14788,7 +14826,7 @@
         <v>1001</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="13"/>
@@ -14798,7 +14836,7 @@
         <v>1010</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C18" s="10"/>
       <c r="H18" s="14"/>
@@ -14809,7 +14847,7 @@
         <v>1011</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H19" s="14"/>
       <c r="I19" s="13"/>
@@ -14819,7 +14857,7 @@
         <v>1100</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H20" s="14"/>
       <c r="I20" s="13"/>
@@ -14829,7 +14867,7 @@
         <v>1101</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H21" s="14"/>
       <c r="I21" s="13"/>
@@ -14839,7 +14877,7 @@
         <v>1110</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H22" s="14"/>
       <c r="I22" s="13"/>
@@ -14849,10 +14887,554 @@
         <v>1111</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H23" s="14"/>
       <c r="I23" s="13"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="H7" s="14"/>
+      <c r="I7" s="13"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="H8" s="14"/>
+      <c r="I8" s="13"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="H9" s="14"/>
+      <c r="I9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="I11" s="14"/>
+      <c r="J11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="I12" s="14"/>
+      <c r="J12" s="13"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="I13" s="14"/>
+      <c r="J13" s="13"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I14" s="14"/>
+      <c r="J14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I15" s="14"/>
+      <c r="J15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I16" s="14"/>
+      <c r="J16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I17" s="14"/>
+      <c r="J17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I18" s="14"/>
+      <c r="J18" s="13"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I19" s="14"/>
+      <c r="J19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="13"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>